<commit_message>
:bee: update plot CT
</commit_message>
<xml_diff>
--- a/data/derived_data/3_CommunityComposition/Dataset_1/ps_rare_16S_D1bis_otu_table.xlsx
+++ b/data/derived_data/3_CommunityComposition/Dataset_1/ps_rare_16S_D1bis_otu_table.xlsx
@@ -12,11 +12,20 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
   <si>
     <t xml:space="preserve"/>
   </si>
   <si>
+    <t xml:space="preserve">MS_086</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_087</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_089</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_090</t>
   </si>
   <si>
@@ -26,6 +35,18 @@
     <t xml:space="preserve">MS_092</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_093</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_095</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_096</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_097</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_099</t>
   </si>
   <si>
@@ -38,6 +59,12 @@
     <t xml:space="preserve">MS_102</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_104</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_117</t>
   </si>
   <si>
@@ -86,6 +113,12 @@
     <t xml:space="preserve">MS_138</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_139</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_140</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_141</t>
   </si>
   <si>
@@ -101,6 +134,9 @@
     <t xml:space="preserve">MS_146</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_152</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_153</t>
   </si>
   <si>
@@ -134,6 +170,9 @@
     <t xml:space="preserve">MS_166</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_167</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_168</t>
   </si>
   <si>
@@ -158,6 +197,9 @@
     <t xml:space="preserve">MS_209</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_210</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_211</t>
   </si>
   <si>
@@ -174,6 +216,15 @@
   </si>
   <si>
     <t xml:space="preserve">MS_220</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_226</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_280</t>
   </si>
   <si>
     <t xml:space="preserve">MS_281</t>
@@ -710,31 +761,82 @@
       <c r="BE1" t="s">
         <v>56</v>
       </c>
+      <c r="BF1" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG1" t="s">
+        <v>58</v>
+      </c>
+      <c r="BH1" t="s">
+        <v>59</v>
+      </c>
+      <c r="BI1" t="s">
+        <v>60</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>61</v>
+      </c>
+      <c r="BK1" t="s">
+        <v>62</v>
+      </c>
+      <c r="BL1" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM1" t="s">
+        <v>64</v>
+      </c>
+      <c r="BN1" t="s">
+        <v>65</v>
+      </c>
+      <c r="BO1" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP1" t="s">
+        <v>67</v>
+      </c>
+      <c r="BQ1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>70</v>
+      </c>
+      <c r="BT1" t="s">
+        <v>71</v>
+      </c>
+      <c r="BU1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BV1" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="B2" t="n">
-        <v>2846</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>2269</v>
       </c>
       <c r="E2" t="n">
-        <v>1860</v>
+        <v>5511</v>
       </c>
       <c r="F2" t="n">
-        <v>1626</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>560</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>794</v>
+        <v>103</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -746,19 +848,19 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>60</v>
+        <v>3935</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>3120</v>
       </c>
       <c r="N2" t="n">
-        <v>767</v>
+        <v>738</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>1900</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>1250</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
@@ -773,16 +875,16 @@
         <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="V2" t="n">
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>1215</v>
       </c>
       <c r="X2" t="n">
-        <v>2748</v>
+        <v>0</v>
       </c>
       <c r="Y2" t="n">
         <v>0</v>
@@ -794,13 +896,13 @@
         <v>0</v>
       </c>
       <c r="AB2" t="n">
-        <v>193</v>
+        <v>0</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
       </c>
       <c r="AD2" t="n">
-        <v>2128</v>
+        <v>0</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
@@ -809,13 +911,13 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>0</v>
+        <v>3706</v>
       </c>
       <c r="AH2" t="n">
-        <v>0</v>
+        <v>1227</v>
       </c>
       <c r="AI2" t="n">
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="AJ2" t="n">
         <v>0</v>
@@ -827,16 +929,16 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>0</v>
+        <v>626</v>
       </c>
       <c r="AN2" t="n">
         <v>0</v>
       </c>
       <c r="AO2" t="n">
-        <v>488</v>
+        <v>1642</v>
       </c>
       <c r="AP2" t="n">
-        <v>0</v>
+        <v>3422</v>
       </c>
       <c r="AQ2" t="n">
         <v>0</v>
@@ -848,10 +950,10 @@
         <v>0</v>
       </c>
       <c r="AT2" t="n">
-        <v>808</v>
+        <v>0</v>
       </c>
       <c r="AU2" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="AV2" t="n">
         <v>0</v>
@@ -872,63 +974,114 @@
         <v>0</v>
       </c>
       <c r="BB2" t="n">
-        <v>0</v>
+        <v>516</v>
       </c>
       <c r="BC2" t="n">
-        <v>2836</v>
+        <v>0</v>
       </c>
       <c r="BD2" t="n">
-        <v>315</v>
+        <v>0</v>
       </c>
       <c r="BE2" t="n">
-        <v>179</v>
+        <v>0</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>937</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>234</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>56</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>153</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>2439</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>3694</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>557</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>524</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="B3" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E3" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F3" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>113</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>111</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="N3" t="n">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="O3" t="n">
-        <v>94</v>
+        <v>305</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
@@ -940,7 +1093,7 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
@@ -952,19 +1105,19 @@
         <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="X3" t="n">
-        <v>0</v>
+        <v>117</v>
       </c>
       <c r="Y3" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="Z3" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="AA3" t="n">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="AB3" t="n">
         <v>0</v>
@@ -973,93 +1126,144 @@
         <v>0</v>
       </c>
       <c r="AD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>9</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>50</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>243</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>211</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>172</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>86</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>65</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>163</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ3" t="n">
+        <v>167</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>531</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>90</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>6</v>
+      </c>
+      <c r="BH3" t="n">
+        <v>10</v>
+      </c>
+      <c r="BI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ3" t="n">
+        <v>61</v>
+      </c>
+      <c r="BR3" t="n">
+        <v>72</v>
+      </c>
+      <c r="BS3" t="n">
         <v>47</v>
       </c>
-      <c r="AE3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>127</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN3" t="n">
-        <v>76</v>
-      </c>
-      <c r="AO3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP3" t="n">
-        <v>111</v>
-      </c>
-      <c r="AQ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR3" t="n">
-        <v>75</v>
-      </c>
-      <c r="AS3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT3" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU3" t="n">
-        <v>2</v>
-      </c>
-      <c r="AV3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC3" t="n">
-        <v>22</v>
-      </c>
-      <c r="BD3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE3" t="n">
-        <v>67</v>
+      <c r="BT3" t="n">
+        <v>28</v>
+      </c>
+      <c r="BU3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV3" t="n">
+        <v>224</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
@@ -1140,10 +1344,10 @@
         <v>0</v>
       </c>
       <c r="AB4" t="n">
-        <v>173</v>
+        <v>0</v>
       </c>
       <c r="AC4" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="AD4" t="n">
         <v>0</v>
@@ -1173,10 +1377,10 @@
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>0</v>
+        <v>616</v>
       </c>
       <c r="AN4" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="AO4" t="n">
         <v>0</v>
@@ -1194,45 +1398,96 @@
         <v>0</v>
       </c>
       <c r="AT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG4" t="n">
         <v>3</v>
       </c>
-      <c r="AU4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE4" t="n">
+      <c r="BH4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ4" t="n">
+        <v>46</v>
+      </c>
+      <c r="BR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="B5" t="n">
         <v>0</v>
@@ -1253,7 +1508,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -1394,39 +1649,90 @@
         <v>0</v>
       </c>
       <c r="BC5" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="BD5" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="BE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS5" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT5" t="n">
+        <v>15</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>129</v>
+      </c>
+      <c r="BV5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>2522</v>
       </c>
       <c r="D6" t="n">
-        <v>765</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>777</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>329</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>4114</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1074</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1435,13 +1741,13 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>701</v>
+        <v>134</v>
       </c>
       <c r="L6" t="n">
-        <v>339</v>
+        <v>1639</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>651</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -1456,16 +1762,16 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>782</v>
+        <v>0</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>0</v>
+        <v>964</v>
       </c>
       <c r="U6" t="n">
-        <v>63</v>
+        <v>355</v>
       </c>
       <c r="V6" t="n">
         <v>0</v>
@@ -1477,13 +1783,13 @@
         <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>243</v>
+        <v>0</v>
       </c>
       <c r="Z6" t="n">
         <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>0</v>
+        <v>934</v>
       </c>
       <c r="AB6" t="n">
         <v>0</v>
@@ -1492,7 +1798,7 @@
         <v>0</v>
       </c>
       <c r="AD6" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="AE6" t="n">
         <v>0</v>
@@ -1510,7 +1816,7 @@
         <v>0</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0</v>
+        <v>871</v>
       </c>
       <c r="AK6" t="n">
         <v>0</v>
@@ -1540,13 +1846,13 @@
         <v>0</v>
       </c>
       <c r="AT6" t="n">
-        <v>225</v>
+        <v>0</v>
       </c>
       <c r="AU6" t="n">
-        <v>86</v>
+        <v>0</v>
       </c>
       <c r="AV6" t="n">
-        <v>2976</v>
+        <v>0</v>
       </c>
       <c r="AW6" t="n">
         <v>0</v>
@@ -1555,66 +1861,117 @@
         <v>0</v>
       </c>
       <c r="AY6" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AZ6" t="n">
-        <v>1399</v>
+        <v>0</v>
       </c>
       <c r="BA6" t="n">
-        <v>676</v>
+        <v>0</v>
       </c>
       <c r="BB6" t="n">
-        <v>127</v>
+        <v>0</v>
       </c>
       <c r="BC6" t="n">
         <v>0</v>
       </c>
       <c r="BD6" t="n">
-        <v>1643</v>
+        <v>0</v>
       </c>
       <c r="BE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>263</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>182</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>6534</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>2203</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>7228</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>2300</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>1184</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>272</v>
+      </c>
+      <c r="BQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR6" t="n">
+        <v>259</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>2874</v>
+      </c>
+      <c r="BV6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>142</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -1713,13 +2070,13 @@
         <v>0</v>
       </c>
       <c r="AT7" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="AU7" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AV7" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AW7" t="n">
         <v>0</v>
@@ -1746,227 +2103,329 @@
         <v>0</v>
       </c>
       <c r="BE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>69</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>29</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>49</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>29</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>2235</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>19893</v>
       </c>
       <c r="G8" t="n">
-        <v>510</v>
+        <v>12115</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>2375</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>2299</v>
+        <v>381</v>
       </c>
       <c r="L8" t="n">
-        <v>2601</v>
+        <v>150</v>
       </c>
       <c r="M8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>1333</v>
+        <v>731</v>
       </c>
       <c r="O8" t="n">
-        <v>708</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>3000</v>
+        <v>2195</v>
       </c>
       <c r="R8" t="n">
-        <v>2218</v>
+        <v>4613</v>
       </c>
       <c r="S8" t="n">
-        <v>3000</v>
+        <v>2740</v>
       </c>
       <c r="T8" t="n">
-        <v>3000</v>
+        <v>3037</v>
       </c>
       <c r="U8" t="n">
-        <v>2937</v>
+        <v>2748</v>
       </c>
       <c r="V8" t="n">
-        <v>3000</v>
+        <v>8993</v>
       </c>
       <c r="W8" t="n">
-        <v>3000</v>
+        <v>2084</v>
       </c>
       <c r="X8" t="n">
-        <v>252</v>
+        <v>990</v>
       </c>
       <c r="Y8" t="n">
-        <v>2511</v>
+        <v>4968</v>
       </c>
       <c r="Z8" t="n">
-        <v>618</v>
+        <v>4744</v>
       </c>
       <c r="AA8" t="n">
-        <v>448</v>
+        <v>2654</v>
       </c>
       <c r="AB8" t="n">
+        <v>4987</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>7281</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>3190</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>3603</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>11474</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>369</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>936</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>755</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>9260</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>1861</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>1069</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>8467</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>5325</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>1048</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>7537</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>3438</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>5601</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>1328</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>12600</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>8778</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>13603</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>7625</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>6481</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>1561</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>2709</v>
+      </c>
+      <c r="BB8" t="n">
         <v>2634</v>
       </c>
-      <c r="AC8" t="n">
-        <v>2968</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>641</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="AF8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="AG8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="AH8" t="n">
-        <v>902</v>
-      </c>
-      <c r="AI8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>752</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>2512</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>1932</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>2872</v>
-      </c>
-      <c r="AR8" t="n">
-        <v>2646</v>
-      </c>
-      <c r="AS8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="AT8" t="n">
-        <v>1702</v>
-      </c>
-      <c r="AU8" t="n">
-        <v>2653</v>
-      </c>
-      <c r="AV8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="AX8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="AY8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ8" t="n">
-        <v>1601</v>
-      </c>
-      <c r="BA8" t="n">
-        <v>2324</v>
-      </c>
-      <c r="BB8" t="n">
-        <v>2873</v>
-      </c>
       <c r="BC8" t="n">
-        <v>0</v>
+        <v>9022</v>
       </c>
       <c r="BD8" t="n">
-        <v>969</v>
+        <v>8224</v>
       </c>
       <c r="BE8" t="n">
-        <v>690</v>
+        <v>2922</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>3155</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>2077</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>4985</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>9887</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>3558</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>2639</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>4225</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>5871</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>1128</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>904</v>
+      </c>
+      <c r="BS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>1634</v>
+      </c>
+      <c r="BV8" t="n">
+        <v>2074</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="B9" t="n">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E9" t="n">
-        <v>229</v>
+        <v>248</v>
       </c>
       <c r="F9" t="n">
-        <v>978</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>413</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>190</v>
+        <v>412</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>514</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>451</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>1874</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>575</v>
       </c>
       <c r="O9" t="n">
-        <v>220</v>
+        <v>411</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
@@ -1978,7 +2437,7 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0</v>
+        <v>626</v>
       </c>
       <c r="T9" t="n">
         <v>0</v>
@@ -1993,7 +2452,7 @@
         <v>0</v>
       </c>
       <c r="X9" t="n">
-        <v>0</v>
+        <v>309</v>
       </c>
       <c r="Y9" t="n">
         <v>0</v>
@@ -2011,7 +2470,7 @@
         <v>0</v>
       </c>
       <c r="AD9" t="n">
-        <v>109</v>
+        <v>0</v>
       </c>
       <c r="AE9" t="n">
         <v>0</v>
@@ -2023,7 +2482,7 @@
         <v>0</v>
       </c>
       <c r="AH9" t="n">
-        <v>1971</v>
+        <v>31</v>
       </c>
       <c r="AI9" t="n">
         <v>0</v>
@@ -2044,10 +2503,10 @@
         <v>0</v>
       </c>
       <c r="AO9" t="n">
-        <v>0</v>
+        <v>786</v>
       </c>
       <c r="AP9" t="n">
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="AQ9" t="n">
         <v>0</v>
@@ -2059,10 +2518,10 @@
         <v>0</v>
       </c>
       <c r="AT9" t="n">
-        <v>31</v>
+        <v>2790</v>
       </c>
       <c r="AU9" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="AV9" t="n">
         <v>0</v>
@@ -2092,12 +2551,63 @@
         <v>0</v>
       </c>
       <c r="BE9" t="n">
-        <v>56</v>
+        <v>0</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>45</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>121</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ9" t="n">
+        <v>254</v>
+      </c>
+      <c r="BR9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV9" t="n">
+        <v>168</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
@@ -2115,10 +2625,10 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>1462</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>1903</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -2136,13 +2646,13 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>818</v>
+        <v>1979</v>
       </c>
       <c r="O10" t="n">
-        <v>1978</v>
+        <v>4623</v>
       </c>
       <c r="P10" t="n">
-        <v>0</v>
+        <v>792</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
@@ -2163,19 +2673,19 @@
         <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>1217</v>
       </c>
       <c r="X10" t="n">
-        <v>0</v>
+        <v>2975</v>
       </c>
       <c r="Y10" t="n">
-        <v>179</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>2302</v>
+        <v>0</v>
       </c>
       <c r="AA10" t="n">
-        <v>2476</v>
+        <v>0</v>
       </c>
       <c r="AB10" t="n">
         <v>0</v>
@@ -2184,7 +2694,7 @@
         <v>0</v>
       </c>
       <c r="AD10" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="AE10" t="n">
         <v>0</v>
@@ -2199,43 +2709,43 @@
         <v>0</v>
       </c>
       <c r="AI10" t="n">
-        <v>0</v>
+        <v>442</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0</v>
+        <v>619</v>
       </c>
       <c r="AK10" t="n">
-        <v>0</v>
+        <v>6732</v>
       </c>
       <c r="AL10" t="n">
-        <v>0</v>
+        <v>5863</v>
       </c>
       <c r="AM10" t="n">
         <v>0</v>
       </c>
       <c r="AN10" t="n">
-        <v>2172</v>
+        <v>0</v>
       </c>
       <c r="AO10" t="n">
         <v>0</v>
       </c>
       <c r="AP10" t="n">
-        <v>957</v>
+        <v>108</v>
       </c>
       <c r="AQ10" t="n">
-        <v>128</v>
+        <v>0</v>
       </c>
       <c r="AR10" t="n">
-        <v>279</v>
+        <v>0</v>
       </c>
       <c r="AS10" t="n">
         <v>0</v>
       </c>
       <c r="AT10" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="AU10" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="AV10" t="n">
         <v>0</v>
@@ -2250,7 +2760,7 @@
         <v>0</v>
       </c>
       <c r="AZ10" t="n">
-        <v>0</v>
+        <v>4315</v>
       </c>
       <c r="BA10" t="n">
         <v>0</v>
@@ -2259,13 +2769,64 @@
         <v>0</v>
       </c>
       <c r="BC10" t="n">
-        <v>134</v>
+        <v>4306</v>
       </c>
       <c r="BD10" t="n">
-        <v>0</v>
+        <v>401</v>
       </c>
       <c r="BE10" t="n">
-        <v>2008</v>
+        <v>311</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>203</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>114</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ10" t="n">
+        <v>194</v>
+      </c>
+      <c r="BR10" t="n">
+        <v>554</v>
+      </c>
+      <c r="BS10" t="n">
+        <v>248</v>
+      </c>
+      <c r="BT10" t="n">
+        <v>174</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV10" t="n">
+        <v>5682</v>
       </c>
     </row>
   </sheetData>

</xml_diff>